<commit_message>
version update und fixed broken example links
</commit_message>
<xml_diff>
--- a/output/StructureDefinition-CustomIdatValues.xlsx
+++ b/output/StructureDefinition-CustomIdatValues.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2025.2.0</t>
+    <t>2026.1.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-06-12</t>
+    <t>2026-02-05</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -96,7 +96,7 @@
     <t>Copyright</t>
   </si>
   <si>
-    <t>Copyright 2020-2025 Unabhängige Treuhandstelle der Universitätsmedizin Greifswald</t>
+    <t>Copyright 2020-2026 Unabhängige Treuhandstelle der Universitätsmedizin Greifswald</t>
   </si>
   <si>
     <t>FHIR Version</t>

</xml_diff>

<commit_message>
fixed examples and several opdef states
</commit_message>
<xml_diff>
--- a/output/StructureDefinition-CustomIdatValues.xlsx
+++ b/output/StructureDefinition-CustomIdatValues.xlsx
@@ -325,9 +325,6 @@
     <t>Element.extension</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>Extension.extension:value1</t>
   </si>
   <si>
@@ -375,6 +372,9 @@
   </si>
   <si>
     <t>Extension.url</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
   <si>
     <t>Extension.extension:value1.value[x]</t>
@@ -1383,39 +1383,39 @@
         <v>79</v>
       </c>
       <c r="AI4" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ4" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AK4" t="s" s="2">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s" s="2">
         <v>90</v>
       </c>
       <c r="C5" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s" s="2">
+        <v>101</v>
+      </c>
+      <c r="F5" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G5" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="H5" t="s" s="2">
         <v>102</v>
-      </c>
-      <c r="D5" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="E5" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="F5" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G5" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H5" t="s" s="2">
-        <v>103</v>
       </c>
       <c r="I5" t="s" s="2">
         <v>21</v>
@@ -1427,10 +1427,10 @@
         <v>92</v>
       </c>
       <c r="L5" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="M5" t="s" s="2">
         <v>104</v>
-      </c>
-      <c r="M5" t="s" s="2">
-        <v>105</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1490,7 +1490,7 @@
         <v>79</v>
       </c>
       <c r="AI5" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ5" t="s" s="2">
         <v>82</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="6" hidden="true">
       <c r="A6" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="B6" t="s" s="2">
         <v>106</v>
-      </c>
-      <c r="B6" t="s" s="2">
-        <v>107</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1604,10 +1604,10 @@
     </row>
     <row r="7" hidden="true">
       <c r="A7" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="B7" t="s" s="2">
         <v>108</v>
-      </c>
-      <c r="B7" t="s" s="2">
-        <v>109</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1636,7 +1636,7 @@
         <v>32</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1696,7 +1696,7 @@
         <v>79</v>
       </c>
       <c r="AI7" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ7" t="s" s="2">
         <v>82</v>
@@ -1707,10 +1707,10 @@
     </row>
     <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="B8" t="s" s="2">
         <v>110</v>
-      </c>
-      <c r="B8" t="s" s="2">
-        <v>111</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1733,16 +1733,16 @@
         <v>21</v>
       </c>
       <c r="K8" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L8" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L8" t="s" s="2">
+      <c r="M8" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M8" t="s" s="2">
+      <c r="N8" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N8" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="Q8" s="2"/>
       <c r="R8" t="s" s="2">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="S8" t="s" s="2">
         <v>21</v>
@@ -1792,22 +1792,22 @@
         <v>21</v>
       </c>
       <c r="AF8" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG8" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH8" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI8" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ8" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK8" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG8" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH8" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI8" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ8" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK8" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="9" hidden="true">
@@ -1904,13 +1904,13 @@
         <v>84</v>
       </c>
       <c r="AI9" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ9" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10">
@@ -1936,7 +1936,7 @@
         <v>84</v>
       </c>
       <c r="H10" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I10" t="s" s="2">
         <v>21</v>
@@ -1951,7 +1951,7 @@
         <v>126</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -2011,7 +2011,7 @@
         <v>79</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ10" t="s" s="2">
         <v>82</v>
@@ -2025,7 +2025,7 @@
         <v>127</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2128,7 +2128,7 @@
         <v>128</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2157,7 +2157,7 @@
         <v>32</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2217,7 +2217,7 @@
         <v>79</v>
       </c>
       <c r="AI12" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ12" t="s" s="2">
         <v>82</v>
@@ -2231,7 +2231,7 @@
         <v>129</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2254,16 +2254,16 @@
         <v>21</v>
       </c>
       <c r="K13" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L13" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L13" t="s" s="2">
+      <c r="M13" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M13" t="s" s="2">
+      <c r="N13" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N13" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2313,22 +2313,22 @@
         <v>21</v>
       </c>
       <c r="AF13" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG13" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH13" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI13" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ13" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK13" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG13" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH13" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI13" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ13" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK13" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="14" hidden="true">
@@ -2425,13 +2425,13 @@
         <v>84</v>
       </c>
       <c r="AI14" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ14" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15">
@@ -2457,7 +2457,7 @@
         <v>84</v>
       </c>
       <c r="H15" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I15" t="s" s="2">
         <v>21</v>
@@ -2472,7 +2472,7 @@
         <v>133</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2532,7 +2532,7 @@
         <v>79</v>
       </c>
       <c r="AI15" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ15" t="s" s="2">
         <v>82</v>
@@ -2546,7 +2546,7 @@
         <v>134</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2649,7 +2649,7 @@
         <v>135</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2678,7 +2678,7 @@
         <v>32</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2738,7 +2738,7 @@
         <v>79</v>
       </c>
       <c r="AI17" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ17" t="s" s="2">
         <v>82</v>
@@ -2752,7 +2752,7 @@
         <v>136</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2775,16 +2775,16 @@
         <v>21</v>
       </c>
       <c r="K18" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L18" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L18" t="s" s="2">
+      <c r="M18" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M18" t="s" s="2">
+      <c r="N18" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -2834,22 +2834,22 @@
         <v>21</v>
       </c>
       <c r="AF18" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG18" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH18" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI18" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ18" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK18" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG18" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH18" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI18" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ18" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK18" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="19" hidden="true">
@@ -2946,13 +2946,13 @@
         <v>84</v>
       </c>
       <c r="AI19" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ19" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20">
@@ -2978,7 +2978,7 @@
         <v>84</v>
       </c>
       <c r="H20" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I20" t="s" s="2">
         <v>21</v>
@@ -2993,7 +2993,7 @@
         <v>140</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -3053,7 +3053,7 @@
         <v>79</v>
       </c>
       <c r="AI20" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ20" t="s" s="2">
         <v>82</v>
@@ -3067,7 +3067,7 @@
         <v>141</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3170,7 +3170,7 @@
         <v>142</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3199,7 +3199,7 @@
         <v>32</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3259,7 +3259,7 @@
         <v>79</v>
       </c>
       <c r="AI22" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ22" t="s" s="2">
         <v>82</v>
@@ -3273,7 +3273,7 @@
         <v>143</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3296,16 +3296,16 @@
         <v>21</v>
       </c>
       <c r="K23" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L23" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L23" t="s" s="2">
+      <c r="M23" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M23" t="s" s="2">
+      <c r="N23" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N23" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -3355,22 +3355,22 @@
         <v>21</v>
       </c>
       <c r="AF23" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG23" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH23" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI23" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ23" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK23" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG23" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH23" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI23" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ23" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK23" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="24" hidden="true">
@@ -3467,13 +3467,13 @@
         <v>84</v>
       </c>
       <c r="AI24" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ24" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25">
@@ -3499,7 +3499,7 @@
         <v>84</v>
       </c>
       <c r="H25" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I25" t="s" s="2">
         <v>21</v>
@@ -3514,7 +3514,7 @@
         <v>147</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3574,7 +3574,7 @@
         <v>79</v>
       </c>
       <c r="AI25" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ25" t="s" s="2">
         <v>82</v>
@@ -3588,7 +3588,7 @@
         <v>148</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -3691,7 +3691,7 @@
         <v>149</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -3720,7 +3720,7 @@
         <v>32</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3780,7 +3780,7 @@
         <v>79</v>
       </c>
       <c r="AI27" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ27" t="s" s="2">
         <v>82</v>
@@ -3794,7 +3794,7 @@
         <v>150</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -3817,16 +3817,16 @@
         <v>21</v>
       </c>
       <c r="K28" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L28" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="M28" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M28" t="s" s="2">
+      <c r="N28" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -3876,22 +3876,22 @@
         <v>21</v>
       </c>
       <c r="AF28" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG28" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH28" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI28" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ28" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK28" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG28" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH28" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI28" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ28" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK28" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="29" hidden="true">
@@ -3988,13 +3988,13 @@
         <v>84</v>
       </c>
       <c r="AI29" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ29" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30">
@@ -4020,7 +4020,7 @@
         <v>84</v>
       </c>
       <c r="H30" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I30" t="s" s="2">
         <v>21</v>
@@ -4035,7 +4035,7 @@
         <v>154</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4095,7 +4095,7 @@
         <v>79</v>
       </c>
       <c r="AI30" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ30" t="s" s="2">
         <v>82</v>
@@ -4109,7 +4109,7 @@
         <v>155</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4212,7 +4212,7 @@
         <v>156</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4241,7 +4241,7 @@
         <v>32</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4301,7 +4301,7 @@
         <v>79</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ32" t="s" s="2">
         <v>82</v>
@@ -4315,7 +4315,7 @@
         <v>157</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4338,16 +4338,16 @@
         <v>21</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L33" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="M33" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M33" t="s" s="2">
+      <c r="N33" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -4397,22 +4397,22 @@
         <v>21</v>
       </c>
       <c r="AF33" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG33" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH33" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI33" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ33" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK33" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG33" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH33" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI33" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ33" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK33" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="34" hidden="true">
@@ -4509,13 +4509,13 @@
         <v>84</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ34" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="35">
@@ -4541,7 +4541,7 @@
         <v>84</v>
       </c>
       <c r="H35" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I35" t="s" s="2">
         <v>21</v>
@@ -4556,7 +4556,7 @@
         <v>161</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -4616,7 +4616,7 @@
         <v>79</v>
       </c>
       <c r="AI35" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ35" t="s" s="2">
         <v>82</v>
@@ -4630,7 +4630,7 @@
         <v>162</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -4733,7 +4733,7 @@
         <v>163</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -4762,7 +4762,7 @@
         <v>32</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -4822,7 +4822,7 @@
         <v>79</v>
       </c>
       <c r="AI37" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ37" t="s" s="2">
         <v>82</v>
@@ -4836,7 +4836,7 @@
         <v>164</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -4859,16 +4859,16 @@
         <v>21</v>
       </c>
       <c r="K38" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L38" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L38" t="s" s="2">
+      <c r="M38" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M38" t="s" s="2">
+      <c r="N38" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N38" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -4918,22 +4918,22 @@
         <v>21</v>
       </c>
       <c r="AF38" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG38" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH38" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI38" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ38" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK38" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG38" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH38" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI38" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ38" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK38" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="39" hidden="true">
@@ -5030,13 +5030,13 @@
         <v>84</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ39" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="40">
@@ -5062,7 +5062,7 @@
         <v>84</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I40" t="s" s="2">
         <v>21</v>
@@ -5077,7 +5077,7 @@
         <v>168</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5137,7 +5137,7 @@
         <v>79</v>
       </c>
       <c r="AI40" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ40" t="s" s="2">
         <v>82</v>
@@ -5151,7 +5151,7 @@
         <v>169</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5254,7 +5254,7 @@
         <v>170</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -5283,7 +5283,7 @@
         <v>32</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -5343,7 +5343,7 @@
         <v>79</v>
       </c>
       <c r="AI42" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ42" t="s" s="2">
         <v>82</v>
@@ -5357,7 +5357,7 @@
         <v>171</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -5380,16 +5380,16 @@
         <v>21</v>
       </c>
       <c r="K43" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L43" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L43" t="s" s="2">
+      <c r="M43" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M43" t="s" s="2">
+      <c r="N43" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
@@ -5439,22 +5439,22 @@
         <v>21</v>
       </c>
       <c r="AF43" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG43" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH43" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI43" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ43" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK43" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG43" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH43" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI43" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ43" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK43" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="44" hidden="true">
@@ -5551,13 +5551,13 @@
         <v>84</v>
       </c>
       <c r="AI44" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ44" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45">
@@ -5583,7 +5583,7 @@
         <v>84</v>
       </c>
       <c r="H45" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I45" t="s" s="2">
         <v>21</v>
@@ -5598,7 +5598,7 @@
         <v>175</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -5658,7 +5658,7 @@
         <v>79</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ45" t="s" s="2">
         <v>82</v>
@@ -5672,7 +5672,7 @@
         <v>176</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -5775,7 +5775,7 @@
         <v>177</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -5804,7 +5804,7 @@
         <v>32</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -5864,7 +5864,7 @@
         <v>79</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>82</v>
@@ -5878,7 +5878,7 @@
         <v>178</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -5901,16 +5901,16 @@
         <v>21</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L48" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L48" t="s" s="2">
+      <c r="M48" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M48" t="s" s="2">
+      <c r="N48" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -5960,22 +5960,22 @@
         <v>21</v>
       </c>
       <c r="AF48" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG48" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH48" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI48" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ48" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK48" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG48" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH48" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI48" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ48" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK48" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="49" hidden="true">
@@ -6072,13 +6072,13 @@
         <v>84</v>
       </c>
       <c r="AI49" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ49" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK49" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="50">
@@ -6104,7 +6104,7 @@
         <v>84</v>
       </c>
       <c r="H50" t="s" s="2">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I50" t="s" s="2">
         <v>21</v>
@@ -6119,7 +6119,7 @@
         <v>182</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -6179,7 +6179,7 @@
         <v>79</v>
       </c>
       <c r="AI50" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ50" t="s" s="2">
         <v>82</v>
@@ -6193,7 +6193,7 @@
         <v>183</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -6296,7 +6296,7 @@
         <v>184</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -6325,7 +6325,7 @@
         <v>32</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -6385,7 +6385,7 @@
         <v>79</v>
       </c>
       <c r="AI52" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ52" t="s" s="2">
         <v>82</v>
@@ -6399,7 +6399,7 @@
         <v>185</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -6422,16 +6422,16 @@
         <v>21</v>
       </c>
       <c r="K53" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L53" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L53" t="s" s="2">
+      <c r="M53" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M53" t="s" s="2">
+      <c r="N53" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N53" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
@@ -6481,22 +6481,22 @@
         <v>21</v>
       </c>
       <c r="AF53" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG53" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH53" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI53" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ53" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK53" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG53" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH53" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI53" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ53" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK53" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="54" hidden="true">
@@ -6593,21 +6593,21 @@
         <v>84</v>
       </c>
       <c r="AI54" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ54" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -6630,16 +6630,16 @@
         <v>21</v>
       </c>
       <c r="K55" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L55" t="s" s="2">
         <v>112</v>
       </c>
-      <c r="L55" t="s" s="2">
+      <c r="M55" t="s" s="2">
         <v>113</v>
       </c>
-      <c r="M55" t="s" s="2">
+      <c r="N55" t="s" s="2">
         <v>114</v>
-      </c>
-      <c r="N55" t="s" s="2">
-        <v>115</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
@@ -6689,22 +6689,22 @@
         <v>21</v>
       </c>
       <c r="AF55" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG55" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AH55" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="AI55" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AJ55" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="AK55" t="s" s="2">
         <v>116</v>
-      </c>
-      <c r="AG55" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH55" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI55" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AJ55" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="AK55" t="s" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="56" hidden="true">
@@ -6801,13 +6801,13 @@
         <v>84</v>
       </c>
       <c r="AI56" t="s" s="2">
-        <v>81</v>
+        <v>21</v>
       </c>
       <c r="AJ56" t="s" s="2">
         <v>123</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>